<commit_message>
Format literature review excel columns and text wrap
</commit_message>
<xml_diff>
--- a/literature/literature_review.xlsx
+++ b/literature/literature_review.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,629 +422,642 @@
   </sheetPr>
   <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Retrieval</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Evaluation</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Main Result</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Limitation</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Our Project Relation</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>**Retrieval-Augmented Generation for Knowledge-Intensive NLP Tasks** *(Lewis et al.)*</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Retrieval-Augmented Generation for Knowledge-Intensive NLP Tasks *(Lewis et al.)*</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Pretrained parametric LLMs suffer from stale internal knowledge and hallucinate factual statements on knowledge-intensive queries.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Combines a parametric sequence-to-sequence model (BART) with a non-parametric dense vector index via RAG-Token and RAG-Sequence formulations.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Natural Questions, WebQuestions, CuratedTREC, MS-MARCO.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>BART-large (generator), BERT-base (retriever).</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Dense Passage Retrieval (DPR) with FAISS Maximum Inner Product Search (MIPS).</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Exact Match (EM), F1 score, and human factual evaluation.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Outperforms purely parametric models with significant reductions in hallucination and higher factual precision on open-domain QA.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Generator still risks hallucinating if the retriever fetches irrelevant or noisy passages.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Establishes the foundational backbone of CiteOrAbstain: conditioning answer generation strictly on retrieved surgical documents.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>**RAGAS: Automated Evaluation of Retrieval Augmented Generation** *(Es et al.)*</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RAGAS: Automated Evaluation of Retrieval Augmented Generation *(Es et al.)*</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Evaluating RAG pipelines end-to-end without expensive, human-annotated ground-truth reference texts is challenging.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Introduces a reference-free evaluation framework measuring isolated sub-components of RAG using LLM-assisted judging.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>WikiEval and public technical QA datasets.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>GPT-3.5-Turbo and GPT-4 (evaluator models).</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Standard dense retriever (HuggingFace / OpenAI embeddings).</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Faithfulness, Answer Relevance, and Context Precision metrics correlated against human judgments.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Achieves high correlation with human domain evaluators, providing scalable, reproducible automated benchmarking.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Dependent on a costly evaluator LLM; lacks specific clinical safety and medical contraindication metrics.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Directly guides the implementation of our automated evaluation script to assess answer faithfulness and context grounding.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>**Enabling Large Language Models to Generate Text with Citations (ALCE)** *(Gao et al.)*</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Enabling Large Language Models to Generate Text with Citations (ALCE) *(Gao et al.)*</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>LLMs generate plausible prose but fail to cite verifiable sources or produce unfaithful/hallucinated citations.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Establishes a formal benchmark and evaluation harness for controllable citation generation across multiple task setups.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>ASQA (ambiguous QA), QAMPARI, ELI5.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>LLaMA, InstructGPT, ChatGPT.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>BM25 (sparse) and GTR (Generalizable T5-based dense retriever).</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Citation Precision, Citation Recall, Fluency, and QA correctness.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Shows that current LLMs frequently produce unsupported claims despite fluent style, requiring explicit citation constraints.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Focuses on general-domain web queries rather than high-stakes clinical refusal requirements.</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Directly corresponds to our core milestone metric: *"Does the cited passage really contain the answer?"* (Citation correctness).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>**Knowing When to Ask and When to Answer: Calibrating LLMs with Abstention** *(Yin et al.)*</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Knowing When to Ask and When to Answer: Calibrating LLMs with Abstention *(Yin et al.)*</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>LLMs output overconfident, incorrect predictions on out-of-distribution or uncertain questions instead of admitting ignorance.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Formulates selective prediction and confidence calibration prompts, allowing models to output an explicit abstention token ("I don't know").</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>CoQA, TriviaQA, SQuAD.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>GPT-3, OPT, T5.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Non-retrieval setting (evaluates raw predictive probability and verbalized confidence).</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Coverage vs. Risk curves, Selective Accuracy, and F1 score.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Abstaining on uncertain questions drastically lowers downstream error rates and improves overall system trustworthiness.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>High abstention thresholds cause over-abstention on answerable, borderline queries.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Provides the mathematical and theoretical justification for abstaining (*"I don't know, please ask your care team"*) when similarity is low.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>**A Survey on Hallucination in Large Language Models: Principles, Taxonomy, Challenges** *(Huang et al.)*</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>A Survey on Hallucination in Large Language Models: Principles, Taxonomy, Challenges *(Huang et al.)*</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Lack of a unified conceptual understanding and categorization of why LLMs produce factually inconsistent statements.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Comprehensive survey classifying hallucination roots across pre-training data, alignment, and decoding stages.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Over 50 benchmark datasets and hallucination detection suites.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>GPT-4, PaLM 2, LLaMA-2, and open-source foundation models.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Multi-paradigm review (dense retrieval, knowledge graphs, web grounding).</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Factual consistency, hallucination rate, semantic entailment metrics.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Concludes that scaling model size alone cannot solve hallucination; external factual grounding (RAG) is mandatory.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Review paper; does not introduce a novel algorithmic retrieval technique.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Provides the theoretical foundation justifying why our assistant must never rely on open generation for medical care.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>**Large Language Models Encode Clinical Knowledge (Med-PaLM)** *(Singhal et al.)*</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Large Language Models Encode Clinical Knowledge (Med-PaLM) *(Singhal et al.)*</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>General-purpose foundation models generate medically ungrounded advice that risks severe clinical harm.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Introduces the MultiMedQA benchmark and physician-curated instruction tuning / reinforcement learning alignment.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>MultiMedQA (MedQA, MedMCQA, PubMedQA, LiveQA, HealthSearchQA).</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>PaLM and Flan-PaLM architectures.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Clinical guidelines index and medical search integration.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Scientific consensus agreement, clinical accuracy, and likelihood of patient harm evaluated by physician panels.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Reaches expert clinician performance thresholds on multiple medical benchmark datasets with verified safety guardrails.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Immense parameter scale makes local deployment infeasible; high operational inference latency.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Theoretical justification for our hard refusal rules: immediate redirection on medication dosing, blood thinners, and emergencies.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>**Retrieval-Augmented Generation for Large Language Models: A Survey** *(Gao et al.)*</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Retrieval-Augmented Generation for Large Language Models: A Survey *(Gao et al.)*</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Naive RAG pipelines suffer from low retrieval precision, context window fragmentation, and generation hallucinations.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Analyzes the evolution from Naive to Advanced and Modular RAG, focusing on chunking, reranking, and indexing.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Public QA and summarization benchmarks.</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>ChatGPT, Claude, LLaMA-3, Mistral.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Dense embeddings, sparse BM25, and hybrid search with cross-encoder rerankers.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Hit Rate, Mean Reciprocal Rank (MRR), BLEU, ROUGE, BERTScore.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Demonstrates that optimal chunk sizing with overlapping windows and vector indexing directly dictates retrieval hit rate.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Survey methodology; does not provide a turnkey domain-specific medical implementation.</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Serves as our engineering reference for document preprocessing (chunk size, overlap) and ChromaDB vector search configuration.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>**Dense Passage Retrieval for Open-Domain Question Answering (DPR)** *(Karpukhin et al.)*</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Dense Passage Retrieval for Open-Domain Question Answering (DPR) *(Karpukhin et al.)*</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Traditional keyword retrieval (BM25) fails to capture semantic synonyms and natural colloquial patient phrasing.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Trains dual-encoder architectures using dense vectors, mapping questions and passages into a shared latent semantic space.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Natural Questions, TriviaQA, WebQuestions, CuratedTREC.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Dual BERT-base encoders.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Dense Passage Retrieval (DPR) indexed via FAISS.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Top-k Retrieval Accuracy (Top-20, Top-100 hit rates).</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Substantially outperforms BM25 on top-k retrieval accuracy by capturing semantic intent rather than exact keyword overlap.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Can miss highly specific, rare medical technical codes where exact token matching is necessary.</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Justifies our architectural choice of sentence-transformer embeddings in ChromaDB to match patient queries with clinical guides.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>**The Over-Refusal Dilemma in Safety-Tuned LLMs** *(Zhang et al.)*</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>The Over-Refusal Dilemma in Safety-Tuned LLMs *(Zhang et al.)*</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Aggressively safety-aligned models frequently over-refuse benign user queries that superficially resemble sensitive concepts.</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Constructs stress-test adversarial benchmarks to quantify the trade-off between user utility and safety constraints.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>XSTest and safety-probe challenge sets.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>GPT-4, Claude-2, LLaMA-2-Chat.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Inference-stage safety filtering and system prompt instructions.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>False Refusal Rate (FRR) and True Safety Violation Rate.</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Demonstrates that overly rigid safety thresholds severely degrade user helpfulness and cause unnecessary refusal spikes.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Evaluates direct conversational alignment rather than vector similarity thresholds in RAG pipelines.</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Theoretical foundation for our Milestone 4 empirical study: analyzing how retrieval thresholds trade correct answers for correct refusals.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>**AttrEval: A Unified Benchmark for Fine-Grained Attributable Text Generation** *(Yue et al.)*</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AttrEval: A Unified Benchmark for Fine-Grained Attributable Text Generation *(Yue et al.)*</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Evaluating whether every single sentence in generated answers is fully attributable to reference documents lacks automation.</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Formulates sentence-level attribution verification using Natural Language Inference (NLI) models across RAG benchmarks.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>AttrEval benchmark suite across 7 underlying datasets.</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>GPT-3.5, Flan-T5, DeBERTa-v3 NLI backbones.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Standard RAG retrieval pipelines.</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Sentence-level attribution precision, recall, and entailment accuracy.</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Granular sentence-level verification successfully pinpoints subtle, partial hallucinations that document-level metrics miss.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Multi-step clinical deductive reasoning occasionally triggers false negative entailment predictions.</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Directly guides our 200-question ground-truth labelling protocol and automated citation verification script.</t>
         </is>

</xml_diff>